<commit_message>
Stand vor Bens-Termin Montag 2026-04-21
- BOM bereinigt (White-Label + Schema-Konsistenz, 4x Suffix -0 nachgezogen)
- Reiner-Scans OCR + Erkenntnisse dokumentiert
- Änderungsprotokoll Teile 1-3 vollständig
- BE-IS-202631 → BE-LS-202603 (offiziell bestätigt, veraltete CSV umbenannt)
- CAD-Standard: Feldname korrigiert, 700er-Systematik belegt
- Offen: B16/B12 Nummernkollision (203) für Reiner

Reviewed-by: Claude (Sonnet)
Co-authored-by: Claude <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/03 Bereiche/WEC/Lieferung/Volker Bens/Lagerschalenhalter Lebensmittelindustrie/2026-04-21 Montag-Session/BOM_bereinigt.xlsx
+++ b/03 Bereiche/WEC/Lieferung/Volker Bens/Lagerschalenhalter Lebensmittelindustrie/2026-04-21 Montag-Session/BOM_bereinigt.xlsx
@@ -1,12 +1,12 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="0" yWindow="0" windowWidth="10000" windowHeight="20000" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="171027" fullCalcOnLoad="1"/>
@@ -623,7 +623,7 @@
       </c>
       <c r="B8" s="1" t="inlineStr">
         <is>
-          <t>BE-LS-202603-200</t>
+          <t>BE-LS-202603-200-0</t>
         </is>
       </c>
       <c r="C8" s="1" t="inlineStr">
@@ -1085,7 +1085,7 @@
       </c>
       <c r="B19" s="1" t="inlineStr">
         <is>
-          <t>BE-LS-202603-204</t>
+          <t>BE-LS-202603-204-0</t>
         </is>
       </c>
       <c r="C19" s="1" t="inlineStr">
@@ -1355,7 +1355,7 @@
       </c>
       <c r="B26" s="1" t="inlineStr">
         <is>
-          <t>BE-LS-202603-200</t>
+          <t>BE-LS-202603-200-0</t>
         </is>
       </c>
       <c r="C26" s="1" t="inlineStr">
@@ -1469,7 +1469,7 @@
       </c>
       <c r="B29" s="1" t="inlineStr">
         <is>
-          <t>BE-LS-202603-200</t>
+          <t>BE-LS-202603-200-0</t>
         </is>
       </c>
       <c r="C29" s="1" t="inlineStr">

</xml_diff>

<commit_message>
fix(bens): Werkstoff 1.44.04 -> 1.4404 + LIESMICH komplettiert
- DIN EN 10027-2 Syntax-Fix in BOM (xlsx+csv, Session + _An_Volker), 12 Zellen je Datei
- LIESMICH.txt um Werkstoff-Angabe + BOM-Hinweise ergaenzt (B16-Konflikt, B11/B12-Duplikat transparent)
- Aenderungsprotokoll Teil 5 dokumentiert Fix und verbleibende Reiner-Entscheidungen
- White-Label-Verify _An_Volker/ weiterhin 0 Treffer

Co-Authored-By: Claude Opus 4.7 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/03 Bereiche/WEC/Lieferung/Volker Bens/Lagerschalenhalter Lebensmittelindustrie/2026-04-21 Montag-Session/BOM_bereinigt.xlsx
+++ b/03 Bereiche/WEC/Lieferung/Volker Bens/Lagerschalenhalter Lebensmittelindustrie/2026-04-21 Montag-Session/BOM_bereinigt.xlsx
@@ -642,7 +642,7 @@
       </c>
       <c r="G8" s="1" t="inlineStr">
         <is>
-          <t>Edelstahl 1.44.04</t>
+          <t>Edelstahl 1.4404</t>
         </is>
       </c>
       <c r="H8" s="1" t="inlineStr"/>
@@ -684,7 +684,7 @@
       </c>
       <c r="G9" s="1" t="inlineStr">
         <is>
-          <t>Edelstahl 1.44.04</t>
+          <t>Edelstahl 1.4404</t>
         </is>
       </c>
       <c r="H9" s="1" t="inlineStr"/>
@@ -726,7 +726,7 @@
       </c>
       <c r="G10" s="1" t="inlineStr">
         <is>
-          <t>Edelstahl 1.44.04</t>
+          <t>Edelstahl 1.4404</t>
         </is>
       </c>
       <c r="H10" s="1" t="inlineStr"/>
@@ -818,7 +818,7 @@
       </c>
       <c r="G12" s="1" t="inlineStr">
         <is>
-          <t>Edelstahl 1.44.04</t>
+          <t>Edelstahl 1.4404</t>
         </is>
       </c>
       <c r="H12" s="1" t="inlineStr"/>
@@ -1020,7 +1020,7 @@
       </c>
       <c r="G17" s="1" t="inlineStr">
         <is>
-          <t>Edelstahl 1.44.04</t>
+          <t>Edelstahl 1.4404</t>
         </is>
       </c>
       <c r="H17" s="1" t="inlineStr"/>
@@ -1062,7 +1062,7 @@
       </c>
       <c r="G18" s="1" t="inlineStr">
         <is>
-          <t>Edelstahl 1.44.04</t>
+          <t>Edelstahl 1.4404</t>
         </is>
       </c>
       <c r="H18" s="1" t="inlineStr"/>
@@ -1142,7 +1142,7 @@
       </c>
       <c r="G20" s="1" t="inlineStr">
         <is>
-          <t>Edelstahl 1.44.04</t>
+          <t>Edelstahl 1.4404</t>
         </is>
       </c>
       <c r="H20" s="1" t="inlineStr"/>
@@ -1184,7 +1184,7 @@
       </c>
       <c r="G21" s="1" t="inlineStr">
         <is>
-          <t>Edelstahl 1.44.04</t>
+          <t>Edelstahl 1.4404</t>
         </is>
       </c>
       <c r="H21" s="1" t="inlineStr"/>
@@ -1332,7 +1332,7 @@
       </c>
       <c r="G25" s="1" t="inlineStr">
         <is>
-          <t>Edelstahl 1.44.04</t>
+          <t>Edelstahl 1.4404</t>
         </is>
       </c>
       <c r="H25" s="1" t="inlineStr"/>
@@ -1374,7 +1374,7 @@
       </c>
       <c r="G26" s="1" t="inlineStr">
         <is>
-          <t>Edelstahl 1.44.04</t>
+          <t>Edelstahl 1.4404</t>
         </is>
       </c>
       <c r="H26" s="1" t="inlineStr"/>
@@ -1446,7 +1446,7 @@
       </c>
       <c r="G28" s="1" t="inlineStr">
         <is>
-          <t>Edelstahl 1.44.04</t>
+          <t>Edelstahl 1.4404</t>
         </is>
       </c>
       <c r="H28" s="1" t="inlineStr"/>
@@ -1488,7 +1488,7 @@
       </c>
       <c r="G29" s="1" t="inlineStr">
         <is>
-          <t>Edelstahl 1.44.04</t>
+          <t>Edelstahl 1.4404</t>
         </is>
       </c>
       <c r="H29" s="1" t="inlineStr"/>

</xml_diff>

<commit_message>
Phase 1.5 + 2.1 code complete — live tests pending
</commit_message>
<xml_diff>
--- a/03 Bereiche/WEC/Lieferung/Volker Bens/Lagerschalenhalter Lebensmittelindustrie/2026-04-21 Montag-Session/BOM_bereinigt.xlsx
+++ b/03 Bereiche/WEC/Lieferung/Volker Bens/Lagerschalenhalter Lebensmittelindustrie/2026-04-21 Montag-Session/BOM_bereinigt.xlsx
@@ -454,7 +454,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N29"/>
+  <dimension ref="A1:N26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelRow="0"/>
   <cols>
     <col width="32" customWidth="1" style="1" min="1" max="3"/>
@@ -712,7 +712,7 @@
       </c>
       <c r="C10" s="1" t="inlineStr">
         <is>
-          <t>Steg_Lagerschalenhalter (~recovered)</t>
+          <t>Steg_Lagerschalenhalter</t>
         </is>
       </c>
       <c r="D10" s="1" t="inlineStr">
@@ -963,7 +963,7 @@
       </c>
       <c r="B16" s="1" t="inlineStr">
         <is>
-          <t>BE-LS-202603-203</t>
+          <t>BE-LS-202603-207-0</t>
         </is>
       </c>
       <c r="C16" s="1" t="inlineStr">
@@ -1043,12 +1043,12 @@
       </c>
       <c r="B18" s="1" t="inlineStr">
         <is>
-          <t>BE-LS-202603-206-0</t>
+          <t>BE-LS-202603-204-0</t>
         </is>
       </c>
       <c r="C18" s="1" t="inlineStr">
         <is>
-          <t>Welle_V1 (~recovered)</t>
+          <t>Welle_V1</t>
         </is>
       </c>
       <c r="D18" s="1" t="inlineStr">
@@ -1123,12 +1123,12 @@
       </c>
       <c r="B20" s="1" t="inlineStr">
         <is>
-          <t>BE-LS-202603-206-0</t>
+          <t>BE-LS-202603-204-0</t>
         </is>
       </c>
       <c r="C20" s="1" t="inlineStr">
         <is>
-          <t>Welle_V1 (~recovered)</t>
+          <t>Welle_V1</t>
         </is>
       </c>
       <c r="D20" s="1" t="inlineStr">
@@ -1283,7 +1283,7 @@
       </c>
       <c r="B24" s="1" t="inlineStr">
         <is>
-          <t>BE-LS-202603-1-0</t>
+          <t>BE-LS-202603-001-0</t>
         </is>
       </c>
       <c r="C24" s="1" t="inlineStr">
@@ -1389,120 +1389,6 @@
       <c r="M26" s="1" t="inlineStr"/>
       <c r="N26" s="1" t="inlineStr"/>
     </row>
-    <row r="27">
-      <c r="A27" s="1" t="inlineStr">
-        <is>
-          <t>12</t>
-        </is>
-      </c>
-      <c r="B27" s="1" t="inlineStr">
-        <is>
-          <t>BE-LS-202603-1-0</t>
-        </is>
-      </c>
-      <c r="C27" s="1" t="inlineStr">
-        <is>
-          <t>Schweißgruppe_Halter</t>
-        </is>
-      </c>
-      <c r="D27" s="1" t="inlineStr"/>
-      <c r="E27" s="1" t="inlineStr"/>
-      <c r="F27" s="1" t="n">
-        <v>2</v>
-      </c>
-      <c r="G27" s="1" t="n"/>
-      <c r="H27" s="1" t="inlineStr"/>
-      <c r="I27" s="1" t="inlineStr"/>
-      <c r="J27" s="1" t="inlineStr"/>
-      <c r="K27" s="1" t="inlineStr"/>
-      <c r="L27" s="1" t="inlineStr"/>
-      <c r="M27" s="1" t="inlineStr"/>
-      <c r="N27" s="1" t="inlineStr"/>
-    </row>
-    <row r="28">
-      <c r="A28" s="1" t="inlineStr">
-        <is>
-          <t>12.1</t>
-        </is>
-      </c>
-      <c r="B28" s="1" t="inlineStr">
-        <is>
-          <t>BE-LS-202603-201-0</t>
-        </is>
-      </c>
-      <c r="C28" s="1" t="inlineStr">
-        <is>
-          <t>Lagerschale</t>
-        </is>
-      </c>
-      <c r="D28" s="1" t="inlineStr">
-        <is>
-          <t>Rundstahl</t>
-        </is>
-      </c>
-      <c r="E28" s="1" t="inlineStr"/>
-      <c r="F28" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="G28" s="1" t="inlineStr">
-        <is>
-          <t>Edelstahl 1.4404</t>
-        </is>
-      </c>
-      <c r="H28" s="1" t="inlineStr"/>
-      <c r="I28" s="1" t="inlineStr"/>
-      <c r="J28" s="1" t="inlineStr">
-        <is>
-          <t>Einzelteil</t>
-        </is>
-      </c>
-      <c r="K28" s="1" t="inlineStr"/>
-      <c r="L28" s="1" t="inlineStr"/>
-      <c r="M28" s="1" t="inlineStr"/>
-      <c r="N28" s="1" t="inlineStr"/>
-    </row>
-    <row r="29">
-      <c r="A29" s="1" t="inlineStr">
-        <is>
-          <t>12.2</t>
-        </is>
-      </c>
-      <c r="B29" s="1" t="inlineStr">
-        <is>
-          <t>BE-LS-202603-200-0</t>
-        </is>
-      </c>
-      <c r="C29" s="1" t="inlineStr">
-        <is>
-          <t>Lagerhalter</t>
-        </is>
-      </c>
-      <c r="D29" s="1" t="inlineStr">
-        <is>
-          <t>Blech 10</t>
-        </is>
-      </c>
-      <c r="E29" s="1" t="inlineStr"/>
-      <c r="F29" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="G29" s="1" t="inlineStr">
-        <is>
-          <t>Edelstahl 1.4404</t>
-        </is>
-      </c>
-      <c r="H29" s="1" t="inlineStr"/>
-      <c r="I29" s="1" t="inlineStr"/>
-      <c r="J29" s="1" t="inlineStr">
-        <is>
-          <t>Einzelteil</t>
-        </is>
-      </c>
-      <c r="K29" s="1" t="inlineStr"/>
-      <c r="L29" s="1" t="inlineStr"/>
-      <c r="M29" s="1" t="inlineStr"/>
-      <c r="N29" s="1" t="inlineStr"/>
-    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="landscape" paperSize="9" scale="100" fitToHeight="1" fitToWidth="1" horizontalDpi="4294967295" verticalDpi="4294967295"/>

</xml_diff>